<commit_message>
Auditoria final-6: custo-hora >= 0, residuos, total bruto de despesas, convenio 0, lookup >= 0, particular obrigatorio, faixa invertida
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
@@ -2445,7 +2445,7 @@
         <v>0.6875</v>
       </c>
       <c r="H5" s="22">
-        <f>IF(A5="","",IF(NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),"faltam as horas faturáveis",C5/F5))))</f>
+        <f>IF(NOT(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;"")),"",IF(A5="","falta o nome",IF(NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),"faltam as horas faturáveis",C5/F5)))))</f>
         <v>54.5454545454546</v>
       </c>
       <c r="I5" s="22">
@@ -2457,7 +2457,7 @@
         <v>117.354419773775</v>
       </c>
       <c r="K5" s="40">
-        <f>IF(AND(A5&lt;&gt;"",OR(NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;""),OR(A5="",NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
         <v>0.6875</v>
       </c>
       <c r="H6" s="22">
-        <f>IF(A6="","",IF(NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),"faltam as horas faturáveis",C6/F6))))</f>
+        <f>IF(NOT(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;"")),"",IF(A6="","falta o nome",IF(NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),"faltam as horas faturáveis",C6/F6)))))</f>
         <v>54.5454545454546</v>
       </c>
       <c r="I6" s="22">
@@ -2503,7 +2503,7 @@
         <v>117.354419773775</v>
       </c>
       <c r="K6" s="40">
-        <f>IF(AND(A6&lt;&gt;"",OR(NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;""),OR(A6="",NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2537,7 +2537,7 @@
         <v>0.5</v>
       </c>
       <c r="H7" s="22">
-        <f>IF(A7="","",IF(NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),"faltam as horas faturáveis",C7/F7))))</f>
+        <f>IF(NOT(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;"")),"",IF(A7="","falta o nome",IF(NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),"faltam as horas faturáveis",C7/F7)))))</f>
         <v>23.3333333333333</v>
       </c>
       <c r="I7" s="22">
@@ -2549,7 +2549,7 @@
         <v>67.0122887864823</v>
       </c>
       <c r="K7" s="40">
-        <f>IF(AND(A7&lt;&gt;"",OR(NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;""),OR(A7="",NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(A8="","",IF(NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),"faltam as horas faturáveis",C8/F8))))</f>
+        <f>IF(NOT(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;"")),"",IF(A8="","falta o nome",IF(NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),"faltam as horas faturáveis",C8/F8)))))</f>
         <v/>
       </c>
       <c r="I8" s="22">
@@ -2577,7 +2577,7 @@
         <v/>
       </c>
       <c r="K8" s="40">
-        <f>IF(AND(A8&lt;&gt;"",OR(NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;""),OR(A8="",NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(A9="","",IF(NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),"faltam as horas faturáveis",C9/F9))))</f>
+        <f>IF(NOT(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;"")),"",IF(A9="","falta o nome",IF(NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),"faltam as horas faturáveis",C9/F9)))))</f>
         <v/>
       </c>
       <c r="I9" s="22">
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="K9" s="40">
-        <f>IF(AND(A9&lt;&gt;"",OR(NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;""),OR(A9="",NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(A10="","",IF(NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),"faltam as horas faturáveis",C10/F10))))</f>
+        <f>IF(NOT(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;"")),"",IF(A10="","falta o nome",IF(NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),"faltam as horas faturáveis",C10/F10)))))</f>
         <v/>
       </c>
       <c r="I10" s="22">
@@ -2633,7 +2633,7 @@
         <v/>
       </c>
       <c r="K10" s="40">
-        <f>IF(AND(A10&lt;&gt;"",OR(NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;""),OR(A10="",NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(A11="","",IF(NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),"faltam as horas faturáveis",C11/F11))))</f>
+        <f>IF(NOT(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;"")),"",IF(A11="","falta o nome",IF(NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),"faltam as horas faturáveis",C11/F11)))))</f>
         <v/>
       </c>
       <c r="I11" s="22">
@@ -2661,7 +2661,7 @@
         <v/>
       </c>
       <c r="K11" s="40">
-        <f>IF(AND(A11&lt;&gt;"",OR(NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;""),OR(A11="",NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(A12="","",IF(NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),"faltam as horas faturáveis",C12/F12))))</f>
+        <f>IF(NOT(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;"")),"",IF(A12="","falta o nome",IF(NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),"faltam as horas faturáveis",C12/F12)))))</f>
         <v/>
       </c>
       <c r="I12" s="22">
@@ -2689,7 +2689,7 @@
         <v/>
       </c>
       <c r="K12" s="40">
-        <f>IF(AND(A12&lt;&gt;"",OR(NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;""),OR(A12="",NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
         <v/>
       </c>
       <c r="H13" s="22">
-        <f>IF(A13="","",IF(NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),"faltam as horas faturáveis",C13/F13))))</f>
+        <f>IF(NOT(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;"")),"",IF(A13="","falta o nome",IF(NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),"faltam as horas faturáveis",C13/F13)))))</f>
         <v/>
       </c>
       <c r="I13" s="22">
@@ -2717,7 +2717,7 @@
         <v/>
       </c>
       <c r="K13" s="40">
-        <f>IF(AND(A13&lt;&gt;"",OR(NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;""),OR(A13="",NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>IF(A14="","",IF(NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),"faltam as horas faturáveis",C14/F14))))</f>
+        <f>IF(NOT(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;"")),"",IF(A14="","falta o nome",IF(NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),"faltam as horas faturáveis",C14/F14)))))</f>
         <v/>
       </c>
       <c r="I14" s="22">
@@ -2745,7 +2745,7 @@
         <v/>
       </c>
       <c r="K14" s="40">
-        <f>IF(AND(A14&lt;&gt;"",OR(NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;""),OR(A14="",NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"))),1,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auditoria final-6: correcoes achadas pela varredura reforcada (custo fixo sem descricao, horas de pessoa incompleta, eco vazio no painel, comparacao com particular negativo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
@@ -1097,7 +1097,7 @@
     </row>
     <row r="6">
       <c r="A6" s="18">
-        <f>IF((SUM(Pessoas!$K$5:$K$14)+IF(ISNUMBER('Custos fixos'!$B$36),0,1))=0,"",IF(IF(ISNUMBER('Custos fixos'!$B$36),0,1)&gt;0,"Atenção: há custo fixo sem valor, com texto ou negativo na aba Custos fixos. ","")&amp;IF(SUM(Pessoas!$K$5:$K$14)&gt;0,"Atenção: "&amp;SUM(Pessoas!$K$5:$K$14)&amp;" pessoa(s) na aba Pessoas com pró-labore, horas faturáveis ou 'já está nos custos fixos?' em branco. ","")&amp;"Custo do mês, custo-hora e hora mínima ficam como 'cadastro incompleto' até você completar: uma soma parcial daria um custo-hora MENOR do que o real.")</f>
+        <f>IF((SUM(Pessoas!$K$5:$K$14)+IF(ISNUMBER('Custos fixos'!$B$36),0,1))=0,"",IF(IF(ISNUMBER('Custos fixos'!$B$36),0,1)&gt;0,"Atenção: há custo fixo sem descrição, sem valor, com texto ou negativo na aba Custos fixos. ","")&amp;IF(SUM(Pessoas!$K$5:$K$14)&gt;0,"Atenção: "&amp;SUM(Pessoas!$K$5:$K$14)&amp;" pessoa(s) na aba Pessoas com pró-labore, horas faturáveis ou 'já está nos custos fixos?' em branco. ","")&amp;"Custo do mês, custo-hora e hora mínima ficam como 'cadastro incompleto' até você completar: uma soma parcial daria um custo-hora MENOR do que o real.")</f>
         <v/>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
         </is>
       </c>
       <c r="B20" s="27">
-        <f>IF(SUMPRODUCT((Pessoas!$A$5:$A$14&lt;&gt;"")*((ISNUMBER(Pessoas!$E$5:$E$14)=FALSE)+ISNUMBER(Pessoas!$E$5:$E$14)*(Pessoas!$E$5:$E$14&lt;0)&gt;0))&gt;0,"faltam horas de trabalho",SUM(Pessoas!$E$5:$E$14))</f>
+        <f>IF((SUM(Pessoas!$K$5:$K$14)+IF(ISNUMBER('Custos fixos'!$B$36),0,1))&gt;0,"cadastro incompleto",IF(SUMPRODUCT((Pessoas!$A$5:$A$14&lt;&gt;"")*((ISNUMBER(Pessoas!$E$5:$E$14)=FALSE)+ISNUMBER(Pessoas!$E$5:$E$14)*(Pessoas!$E$5:$E$14&lt;0)&gt;0))&gt;0,"faltam horas de trabalho",SUM(Pessoas!$E$5:$E$14)))</f>
         <v>440</v>
       </c>
       <c r="C20" s="23" t="inlineStr">
@@ -1409,7 +1409,7 @@
         <v>Marina Ferraz</v>
       </c>
       <c r="B26" s="21" t="str">
-        <f>IF(Pessoas!$A$5="","",Pessoas!$B$5)</f>
+        <f>IF(OR(Pessoas!$A$5="",Pessoas!$B$5=""),"",Pessoas!$B$5)</f>
         <v>Sócia · cível e empresarial</v>
       </c>
       <c r="C26" s="27">
@@ -1439,7 +1439,7 @@
         <v>Rafael Lima</v>
       </c>
       <c r="B27" s="21" t="str">
-        <f>IF(Pessoas!$A$6="","",Pessoas!$B$6)</f>
+        <f>IF(OR(Pessoas!$A$6="",Pessoas!$B$6=""),"",Pessoas!$B$6)</f>
         <v>Sócio · trabalhista e previdenciário</v>
       </c>
       <c r="C27" s="27">
@@ -1469,7 +1469,7 @@
         <v>Júlia Prado</v>
       </c>
       <c r="B28" s="21" t="str">
-        <f>IF(Pessoas!$A$7="","",Pessoas!$B$7)</f>
+        <f>IF(OR(Pessoas!$A$7="",Pessoas!$B$7=""),"",Pessoas!$B$7)</f>
         <v>Estagiária</v>
       </c>
       <c r="C28" s="27">
@@ -1499,7 +1499,7 @@
         <v/>
       </c>
       <c r="B29" s="21">
-        <f>IF(Pessoas!$A$8="","",Pessoas!$B$8)</f>
+        <f>IF(OR(Pessoas!$A$8="",Pessoas!$B$8=""),"",Pessoas!$B$8)</f>
         <v/>
       </c>
       <c r="C29" s="27">
@@ -1529,7 +1529,7 @@
         <v/>
       </c>
       <c r="B30" s="21">
-        <f>IF(Pessoas!$A$9="","",Pessoas!$B$9)</f>
+        <f>IF(OR(Pessoas!$A$9="",Pessoas!$B$9=""),"",Pessoas!$B$9)</f>
         <v/>
       </c>
       <c r="C30" s="27">
@@ -1559,7 +1559,7 @@
         <v/>
       </c>
       <c r="B31" s="21">
-        <f>IF(Pessoas!$A$10="","",Pessoas!$B$10)</f>
+        <f>IF(OR(Pessoas!$A$10="",Pessoas!$B$10=""),"",Pessoas!$B$10)</f>
         <v/>
       </c>
       <c r="C31" s="27">
@@ -1589,7 +1589,7 @@
         <v/>
       </c>
       <c r="B32" s="21">
-        <f>IF(Pessoas!$A$11="","",Pessoas!$B$11)</f>
+        <f>IF(OR(Pessoas!$A$11="",Pessoas!$B$11=""),"",Pessoas!$B$11)</f>
         <v/>
       </c>
       <c r="C32" s="27">
@@ -1619,7 +1619,7 @@
         <v/>
       </c>
       <c r="B33" s="21">
-        <f>IF(Pessoas!$A$12="","",Pessoas!$B$12)</f>
+        <f>IF(OR(Pessoas!$A$12="",Pessoas!$B$12=""),"",Pessoas!$B$12)</f>
         <v/>
       </c>
       <c r="C33" s="27">
@@ -1649,7 +1649,7 @@
         <v/>
       </c>
       <c r="B34" s="21">
-        <f>IF(Pessoas!$A$13="","",Pessoas!$B$13)</f>
+        <f>IF(OR(Pessoas!$A$13="",Pessoas!$B$13=""),"",Pessoas!$B$13)</f>
         <v/>
       </c>
       <c r="C34" s="27">
@@ -1679,7 +1679,7 @@
         <v/>
       </c>
       <c r="B35" s="21">
-        <f>IF(Pessoas!$A$14="","",Pessoas!$B$14)</f>
+        <f>IF(OR(Pessoas!$A$14="",Pessoas!$B$14=""),"",Pessoas!$B$14)</f>
         <v/>
       </c>
       <c r="C35" s="27">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="B36" s="26">
-        <f>IF(SUMPRODUCT(((A5:A34&lt;&gt;"")+(B5:B34&lt;&gt;"")&gt;0)*((ISNUMBER(B5:B34)=FALSE)+ISNUMBER(B5:B34)*(B5:B34&lt;0)&gt;0))&gt;0,"custo fixo sem valor numérico ou negativo",SUM(B5:B34))</f>
+        <f>IF(SUMPRODUCT(((A5:A34&lt;&gt;"")+(B5:B34&lt;&gt;"")&gt;0)*((A5:A34="")+(ISNUMBER(B5:B34)=FALSE)+ISNUMBER(B5:B34)*(B5:B34&lt;0)&gt;0))&gt;0,"custo fixo sem descrição, sem valor numérico ou negativo",SUM(B5:B34))</f>
         <v>6500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auditoria final-7: excecao do convenio 0 so na linha Retorno (F7-G01) e horas faturaveis acima das de trabalho como pendencia (F7-M01)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0146uBo6FVJ2cyEehyP8rK61
</commit_message>
<xml_diff>
--- a/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
+++ b/projetos/gestao-ia-planilhas/produto/kit-advogados/05-custo-hora.xlsx
@@ -1097,7 +1097,7 @@
     </row>
     <row r="6">
       <c r="A6" s="18">
-        <f>IF((SUM(Pessoas!$K$5:$K$14)+IF(ISNUMBER('Custos fixos'!$B$36),0,1))=0,"",IF(IF(ISNUMBER('Custos fixos'!$B$36),0,1)&gt;0,"Atenção: há custo fixo sem descrição, sem valor, com texto ou negativo na aba Custos fixos. ","")&amp;IF(SUM(Pessoas!$K$5:$K$14)&gt;0,"Atenção: "&amp;SUM(Pessoas!$K$5:$K$14)&amp;" pessoa(s) na aba Pessoas com pró-labore, horas faturáveis ou 'já está nos custos fixos?' em branco. ","")&amp;"Custo do mês, custo-hora e hora mínima ficam como 'cadastro incompleto' até você completar: uma soma parcial daria um custo-hora MENOR do que o real.")</f>
+        <f>IF((SUM(Pessoas!$K$5:$K$14)+IF(ISNUMBER('Custos fixos'!$B$36),0,1))=0,"",IF(IF(ISNUMBER('Custos fixos'!$B$36),0,1)&gt;0,"Atenção: há custo fixo sem descrição, sem valor, com texto ou negativo na aba Custos fixos. ","")&amp;IF(SUM(Pessoas!$K$5:$K$14)&gt;0,"Atenção: "&amp;SUM(Pessoas!$K$5:$K$14)&amp;" pessoa(s) na aba Pessoas com pró-labore, horas faturáveis ou 'já está nos custos fixos?' em branco, ou com horas faturáveis acima das horas de trabalho. ","")&amp;"Custo do mês, custo-hora e hora mínima ficam como 'cadastro incompleto' até você completar: uma soma parcial daria um custo-hora MENOR do que o real.")</f>
         <v/>
       </c>
     </row>
@@ -2441,11 +2441,11 @@
         <v>110</v>
       </c>
       <c r="G5" s="28">
-        <f>IF(OR(A5="",NOT(IF(ISNUMBER(E5),E5&gt;0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;=0,FALSE))),"",F5/E5)</f>
+        <f>IF(OR(A5="",NOT(IF(ISNUMBER(E5),E5&gt;0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;=0,FALSE))),"",IF(F5&gt;E5,"faturáveis &gt; trabalho",F5/E5))</f>
         <v>0.6875</v>
       </c>
       <c r="H5" s="22">
-        <f>IF(NOT(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;"")),"",IF(A5="","falta o nome",IF(NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),"faltam as horas faturáveis",C5/F5)))))</f>
+        <f>IF(NOT(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;"")),"",IF(A5="","falta o nome",IF(NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E5),F5&gt;E5),"faturáveis acima das horas de trabalho",C5/F5))))))</f>
         <v>54.5454545454546</v>
       </c>
       <c r="I5" s="22">
@@ -2457,7 +2457,7 @@
         <v>117.354419773775</v>
       </c>
       <c r="K5" s="40">
-        <f>IF(AND(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;""),OR(A5="",NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A5&lt;&gt;"",B5&lt;&gt;"",C5&lt;&gt;"",D5&lt;&gt;"",E5&lt;&gt;"",F5&lt;&gt;""),OR(A5="",NOT(IF(ISNUMBER(C5),C5&gt;=0,FALSE)),NOT(IF(ISNUMBER(F5),F5&gt;0,FALSE)),AND(D5&lt;&gt;"Sim",D5&lt;&gt;"Não"),AND(ISNUMBER(E5),ISNUMBER(F5),N(F5)&gt;N(E5)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2487,11 +2487,11 @@
         <v>110</v>
       </c>
       <c r="G6" s="28">
-        <f>IF(OR(A6="",NOT(IF(ISNUMBER(E6),E6&gt;0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;=0,FALSE))),"",F6/E6)</f>
+        <f>IF(OR(A6="",NOT(IF(ISNUMBER(E6),E6&gt;0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;=0,FALSE))),"",IF(F6&gt;E6,"faturáveis &gt; trabalho",F6/E6))</f>
         <v>0.6875</v>
       </c>
       <c r="H6" s="22">
-        <f>IF(NOT(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;"")),"",IF(A6="","falta o nome",IF(NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),"faltam as horas faturáveis",C6/F6)))))</f>
+        <f>IF(NOT(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;"")),"",IF(A6="","falta o nome",IF(NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E6),F6&gt;E6),"faturáveis acima das horas de trabalho",C6/F6))))))</f>
         <v>54.5454545454546</v>
       </c>
       <c r="I6" s="22">
@@ -2503,7 +2503,7 @@
         <v>117.354419773775</v>
       </c>
       <c r="K6" s="40">
-        <f>IF(AND(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;""),OR(A6="",NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A6&lt;&gt;"",B6&lt;&gt;"",C6&lt;&gt;"",D6&lt;&gt;"",E6&lt;&gt;"",F6&lt;&gt;""),OR(A6="",NOT(IF(ISNUMBER(C6),C6&gt;=0,FALSE)),NOT(IF(ISNUMBER(F6),F6&gt;0,FALSE)),AND(D6&lt;&gt;"Sim",D6&lt;&gt;"Não"),AND(ISNUMBER(E6),ISNUMBER(F6),N(F6)&gt;N(E6)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2533,11 +2533,11 @@
         <v>60</v>
       </c>
       <c r="G7" s="28">
-        <f>IF(OR(A7="",NOT(IF(ISNUMBER(E7),E7&gt;0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;=0,FALSE))),"",F7/E7)</f>
+        <f>IF(OR(A7="",NOT(IF(ISNUMBER(E7),E7&gt;0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;=0,FALSE))),"",IF(F7&gt;E7,"faturáveis &gt; trabalho",F7/E7))</f>
         <v>0.5</v>
       </c>
       <c r="H7" s="22">
-        <f>IF(NOT(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;"")),"",IF(A7="","falta o nome",IF(NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),"faltam as horas faturáveis",C7/F7)))))</f>
+        <f>IF(NOT(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;"")),"",IF(A7="","falta o nome",IF(NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E7),F7&gt;E7),"faturáveis acima das horas de trabalho",C7/F7))))))</f>
         <v>23.3333333333333</v>
       </c>
       <c r="I7" s="22">
@@ -2549,7 +2549,7 @@
         <v>67.0122887864823</v>
       </c>
       <c r="K7" s="40">
-        <f>IF(AND(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;""),OR(A7="",NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A7&lt;&gt;"",B7&lt;&gt;"",C7&lt;&gt;"",D7&lt;&gt;"",E7&lt;&gt;"",F7&lt;&gt;""),OR(A7="",NOT(IF(ISNUMBER(C7),C7&gt;=0,FALSE)),NOT(IF(ISNUMBER(F7),F7&gt;0,FALSE)),AND(D7&lt;&gt;"Sim",D7&lt;&gt;"Não"),AND(ISNUMBER(E7),ISNUMBER(F7),N(F7)&gt;N(E7)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2561,11 +2561,11 @@
       <c r="E8" s="39" t="n"/>
       <c r="F8" s="39" t="n"/>
       <c r="G8" s="28">
-        <f>IF(OR(A8="",NOT(IF(ISNUMBER(E8),E8&gt;0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;=0,FALSE))),"",F8/E8)</f>
+        <f>IF(OR(A8="",NOT(IF(ISNUMBER(E8),E8&gt;0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;=0,FALSE))),"",IF(F8&gt;E8,"faturáveis &gt; trabalho",F8/E8))</f>
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(NOT(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;"")),"",IF(A8="","falta o nome",IF(NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),"faltam as horas faturáveis",C8/F8)))))</f>
+        <f>IF(NOT(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;"")),"",IF(A8="","falta o nome",IF(NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E8),F8&gt;E8),"faturáveis acima das horas de trabalho",C8/F8))))))</f>
         <v/>
       </c>
       <c r="I8" s="22">
@@ -2577,7 +2577,7 @@
         <v/>
       </c>
       <c r="K8" s="40">
-        <f>IF(AND(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;""),OR(A8="",NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A8&lt;&gt;"",B8&lt;&gt;"",C8&lt;&gt;"",D8&lt;&gt;"",E8&lt;&gt;"",F8&lt;&gt;""),OR(A8="",NOT(IF(ISNUMBER(C8),C8&gt;=0,FALSE)),NOT(IF(ISNUMBER(F8),F8&gt;0,FALSE)),AND(D8&lt;&gt;"Sim",D8&lt;&gt;"Não"),AND(ISNUMBER(E8),ISNUMBER(F8),N(F8)&gt;N(E8)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2589,11 +2589,11 @@
       <c r="E9" s="39" t="n"/>
       <c r="F9" s="39" t="n"/>
       <c r="G9" s="28">
-        <f>IF(OR(A9="",NOT(IF(ISNUMBER(E9),E9&gt;0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;=0,FALSE))),"",F9/E9)</f>
+        <f>IF(OR(A9="",NOT(IF(ISNUMBER(E9),E9&gt;0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;=0,FALSE))),"",IF(F9&gt;E9,"faturáveis &gt; trabalho",F9/E9))</f>
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(NOT(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;"")),"",IF(A9="","falta o nome",IF(NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),"faltam as horas faturáveis",C9/F9)))))</f>
+        <f>IF(NOT(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;"")),"",IF(A9="","falta o nome",IF(NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E9),F9&gt;E9),"faturáveis acima das horas de trabalho",C9/F9))))))</f>
         <v/>
       </c>
       <c r="I9" s="22">
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="K9" s="40">
-        <f>IF(AND(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;""),OR(A9="",NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A9&lt;&gt;"",B9&lt;&gt;"",C9&lt;&gt;"",D9&lt;&gt;"",E9&lt;&gt;"",F9&lt;&gt;""),OR(A9="",NOT(IF(ISNUMBER(C9),C9&gt;=0,FALSE)),NOT(IF(ISNUMBER(F9),F9&gt;0,FALSE)),AND(D9&lt;&gt;"Sim",D9&lt;&gt;"Não"),AND(ISNUMBER(E9),ISNUMBER(F9),N(F9)&gt;N(E9)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2617,11 +2617,11 @@
       <c r="E10" s="39" t="n"/>
       <c r="F10" s="39" t="n"/>
       <c r="G10" s="28">
-        <f>IF(OR(A10="",NOT(IF(ISNUMBER(E10),E10&gt;0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;=0,FALSE))),"",F10/E10)</f>
+        <f>IF(OR(A10="",NOT(IF(ISNUMBER(E10),E10&gt;0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;=0,FALSE))),"",IF(F10&gt;E10,"faturáveis &gt; trabalho",F10/E10))</f>
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(NOT(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;"")),"",IF(A10="","falta o nome",IF(NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),"faltam as horas faturáveis",C10/F10)))))</f>
+        <f>IF(NOT(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;"")),"",IF(A10="","falta o nome",IF(NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E10),F10&gt;E10),"faturáveis acima das horas de trabalho",C10/F10))))))</f>
         <v/>
       </c>
       <c r="I10" s="22">
@@ -2633,7 +2633,7 @@
         <v/>
       </c>
       <c r="K10" s="40">
-        <f>IF(AND(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;""),OR(A10="",NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A10&lt;&gt;"",B10&lt;&gt;"",C10&lt;&gt;"",D10&lt;&gt;"",E10&lt;&gt;"",F10&lt;&gt;""),OR(A10="",NOT(IF(ISNUMBER(C10),C10&gt;=0,FALSE)),NOT(IF(ISNUMBER(F10),F10&gt;0,FALSE)),AND(D10&lt;&gt;"Sim",D10&lt;&gt;"Não"),AND(ISNUMBER(E10),ISNUMBER(F10),N(F10)&gt;N(E10)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2645,11 +2645,11 @@
       <c r="E11" s="39" t="n"/>
       <c r="F11" s="39" t="n"/>
       <c r="G11" s="28">
-        <f>IF(OR(A11="",NOT(IF(ISNUMBER(E11),E11&gt;0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;=0,FALSE))),"",F11/E11)</f>
+        <f>IF(OR(A11="",NOT(IF(ISNUMBER(E11),E11&gt;0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;=0,FALSE))),"",IF(F11&gt;E11,"faturáveis &gt; trabalho",F11/E11))</f>
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(NOT(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;"")),"",IF(A11="","falta o nome",IF(NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),"faltam as horas faturáveis",C11/F11)))))</f>
+        <f>IF(NOT(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;"")),"",IF(A11="","falta o nome",IF(NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E11),F11&gt;E11),"faturáveis acima das horas de trabalho",C11/F11))))))</f>
         <v/>
       </c>
       <c r="I11" s="22">
@@ -2661,7 +2661,7 @@
         <v/>
       </c>
       <c r="K11" s="40">
-        <f>IF(AND(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;""),OR(A11="",NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A11&lt;&gt;"",B11&lt;&gt;"",C11&lt;&gt;"",D11&lt;&gt;"",E11&lt;&gt;"",F11&lt;&gt;""),OR(A11="",NOT(IF(ISNUMBER(C11),C11&gt;=0,FALSE)),NOT(IF(ISNUMBER(F11),F11&gt;0,FALSE)),AND(D11&lt;&gt;"Sim",D11&lt;&gt;"Não"),AND(ISNUMBER(E11),ISNUMBER(F11),N(F11)&gt;N(E11)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2673,11 +2673,11 @@
       <c r="E12" s="39" t="n"/>
       <c r="F12" s="39" t="n"/>
       <c r="G12" s="28">
-        <f>IF(OR(A12="",NOT(IF(ISNUMBER(E12),E12&gt;0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;=0,FALSE))),"",F12/E12)</f>
+        <f>IF(OR(A12="",NOT(IF(ISNUMBER(E12),E12&gt;0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;=0,FALSE))),"",IF(F12&gt;E12,"faturáveis &gt; trabalho",F12/E12))</f>
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(NOT(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;"")),"",IF(A12="","falta o nome",IF(NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),"faltam as horas faturáveis",C12/F12)))))</f>
+        <f>IF(NOT(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;"")),"",IF(A12="","falta o nome",IF(NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E12),F12&gt;E12),"faturáveis acima das horas de trabalho",C12/F12))))))</f>
         <v/>
       </c>
       <c r="I12" s="22">
@@ -2689,7 +2689,7 @@
         <v/>
       </c>
       <c r="K12" s="40">
-        <f>IF(AND(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;""),OR(A12="",NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A12&lt;&gt;"",B12&lt;&gt;"",C12&lt;&gt;"",D12&lt;&gt;"",E12&lt;&gt;"",F12&lt;&gt;""),OR(A12="",NOT(IF(ISNUMBER(C12),C12&gt;=0,FALSE)),NOT(IF(ISNUMBER(F12),F12&gt;0,FALSE)),AND(D12&lt;&gt;"Sim",D12&lt;&gt;"Não"),AND(ISNUMBER(E12),ISNUMBER(F12),N(F12)&gt;N(E12)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2701,11 +2701,11 @@
       <c r="E13" s="39" t="n"/>
       <c r="F13" s="39" t="n"/>
       <c r="G13" s="28">
-        <f>IF(OR(A13="",NOT(IF(ISNUMBER(E13),E13&gt;0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;=0,FALSE))),"",F13/E13)</f>
+        <f>IF(OR(A13="",NOT(IF(ISNUMBER(E13),E13&gt;0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;=0,FALSE))),"",IF(F13&gt;E13,"faturáveis &gt; trabalho",F13/E13))</f>
         <v/>
       </c>
       <c r="H13" s="22">
-        <f>IF(NOT(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;"")),"",IF(A13="","falta o nome",IF(NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),"faltam as horas faturáveis",C13/F13)))))</f>
+        <f>IF(NOT(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;"")),"",IF(A13="","falta o nome",IF(NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E13),F13&gt;E13),"faturáveis acima das horas de trabalho",C13/F13))))))</f>
         <v/>
       </c>
       <c r="I13" s="22">
@@ -2717,7 +2717,7 @@
         <v/>
       </c>
       <c r="K13" s="40">
-        <f>IF(AND(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;""),OR(A13="",NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A13&lt;&gt;"",B13&lt;&gt;"",C13&lt;&gt;"",D13&lt;&gt;"",E13&lt;&gt;"",F13&lt;&gt;""),OR(A13="",NOT(IF(ISNUMBER(C13),C13&gt;=0,FALSE)),NOT(IF(ISNUMBER(F13),F13&gt;0,FALSE)),AND(D13&lt;&gt;"Sim",D13&lt;&gt;"Não"),AND(ISNUMBER(E13),ISNUMBER(F13),N(F13)&gt;N(E13)))),1,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2729,11 +2729,11 @@
       <c r="E14" s="39" t="n"/>
       <c r="F14" s="39" t="n"/>
       <c r="G14" s="28">
-        <f>IF(OR(A14="",NOT(IF(ISNUMBER(E14),E14&gt;0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;=0,FALSE))),"",F14/E14)</f>
+        <f>IF(OR(A14="",NOT(IF(ISNUMBER(E14),E14&gt;0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;=0,FALSE))),"",IF(F14&gt;E14,"faturáveis &gt; trabalho",F14/E14))</f>
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>IF(NOT(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;"")),"",IF(A14="","falta o nome",IF(NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),"faltam as horas faturáveis",C14/F14)))))</f>
+        <f>IF(NOT(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;"")),"",IF(A14="","falta o nome",IF(NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),"falta o pró-labore",IF(AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"),"falta: já está nos custos fixos?",IF(NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),"faltam as horas faturáveis",IF(AND(ISNUMBER(E14),F14&gt;E14),"faturáveis acima das horas de trabalho",C14/F14))))))</f>
         <v/>
       </c>
       <c r="I14" s="22">
@@ -2745,7 +2745,7 @@
         <v/>
       </c>
       <c r="K14" s="40">
-        <f>IF(AND(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;""),OR(A14="",NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"))),1,0)</f>
+        <f>IF(AND(OR(A14&lt;&gt;"",B14&lt;&gt;"",C14&lt;&gt;"",D14&lt;&gt;"",E14&lt;&gt;"",F14&lt;&gt;""),OR(A14="",NOT(IF(ISNUMBER(C14),C14&gt;=0,FALSE)),NOT(IF(ISNUMBER(F14),F14&gt;0,FALSE)),AND(D14&lt;&gt;"Sim",D14&lt;&gt;"Não"),AND(ISNUMBER(E14),ISNUMBER(F14),N(F14)&gt;N(E14)))),1,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>